<commit_message>
feat: unified observability package (rag/observability/)
Replace rag/tools/langfuse.py with config-driven rag/observability/ package:
- ObservabilityConfig dataclass + preset factories (prod, probe, benchmark, chunking)
- create_trace/finalize_trace lifecycle using Langfuse SDK v4 start_observation
- Declarative eval block system with retry + failure scoring (-1)
- 4 RAGAS blocks: faithfulness, answer_relevancy, context_precision, context_recall
- Standardize all @observe spans to dotted-lowercase (pipeline.router, pipeline.generator, etc.)
- Add cache_hit=true span annotations on router/retrieval cache hits
- Rewrite all callers (app.py, run_probe, run_benchmark, eval_chunking)
- Delete Gate 2, route_retrieve_rerank, router_order dead code

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tamu_data/evals/golden_sets/golden_20260411_v1_reworked6.xlsx
+++ b/tamu_data/evals/golden_sets/golden_20260411_v1_reworked6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,16 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>run:golden_20260411_v1_reworked6_20260412_20260412_102529</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>run:flash_lite_threshold035_20260417_20260417_160416</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>run:reworked6_flash_lite_20260417_20260417_161027</t>
         </is>
       </c>
     </row>
@@ -485,6 +495,16 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>CSCE 608 §? 0.68, CSCE 605 §? 0.67, ISEN 620 §? 0.66, CSCE 614 §? 0.66, CSCE 635 §? 0.64, CSCE 713 §? 0.64, CSCE 681 §? 0.63, CSCE 681 §? 0.62, CSCE 629 §? 0.61, ISEN 620 §? 0.61</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CSCE 605 §? 0.68, CSCE 681 §? 0.63, CSCE 713 §? 0.63, CSCE 629 §? 0.62, CSCE 681 §? 0.59, CSCE 652 §? 0.59, CSCE 614 §? 0.59, ISEN 620 §? 0.59, CSCE 635 §? 0.57, ISEN 620 §? 0.57</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>CSCE 605 §? 0.68, CSCE 681 §? 0.63, CSCE 713 §? 0.63, CSCE 629 §? 0.62, CSCE 681 §? 0.59, CSCE 652 §? 0.59, CSCE 614 §? 0.59, ISEN 620 §? 0.59, CSCE 635 §? 0.57, ISEN 620 §? 0.57</t>
         </is>
       </c>
     </row>
@@ -526,6 +546,16 @@
           <t>CSCE 638 §? 0.73, CSCE 670 §? 0.67, CSCE 641 §? 0.55, CSCE 633 §? 0.51, CSCE 726 §? 0.50, CSCE 726 §? 0.50, CSCE 605 §? 0.50, CSCE 726 §? 0.49, CSCE 665 §? 0.49, CSCE 638 §? 0.47</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CSCE 638 §? 0.72, CSCE 670 §? 0.61</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CSCE 638 §? 0.72, CSCE 670 §? 0.61</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -557,6 +587,16 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>CSCE 632 §? 0.73, CSCE 624 §? 0.71, CSCE 633 §? 0.68, CSCE 614 §? 0.68, CSCE 624 §? 0.66, CSCE 726 §? 0.66, CSCE 641 §? 0.63, CSCE 748 §? 0.62, CSCE 670 §? 0.61, CSCE 605 §? 0.61</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>CSCE 726 §? 0.70, CSCE 624 §? 0.68, CSCE 632 §? 0.68, CSCE 624 §? 0.67, CSCE 635 §? 0.67, CSCE 665 §? 0.67, CSCE 726 §? 0.63, CSCE 726 §? 0.61, CSCE 633 §? 0.59, CSCE 633 §? 0.59</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CSCE 726 §? 0.70, CSCE 624 §? 0.68, CSCE 632 §? 0.68, CSCE 624 §? 0.67, CSCE 635 §? 0.67, CSCE 665 §? 0.67, CSCE 726 §? 0.63, CSCE 726 §? 0.61, CSCE 633 §? 0.59, CSCE 633 §? 0.59</t>
         </is>
       </c>
     </row>
@@ -597,6 +637,16 @@
           <t>CSCE 611 §? 0.59, CSCE 611 §? 0.51, CSCE 611 §? 0.50, CSCE 611 §? 0.43, CSCE 611 §? 0.25</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.54, CSCE 611 §? 0.51, CSCE 611 §? 0.51, CSCE 611 §? 0.46</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.54, CSCE 611 §? 0.51, CSCE 611 §? 0.51, CSCE 611 §? 0.46</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -626,6 +676,16 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>CSCE 611 §? 0.68, CSCE 611 §? 0.59, CSCE 611 §? 0.39, CSCE 611 §? 0.25, CSCE 611 §? 0.17</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.67, CSCE 611 §? 0.65</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.67, CSCE 611 §? 0.65</t>
         </is>
       </c>
     </row>

</xml_diff>